<commit_message>
making imports lazy for better testing
</commit_message>
<xml_diff>
--- a/monet/tests/TestData/control/feedback_test_db.xlsx
+++ b/monet/tests/TestData/control/feedback_test_db.xlsx
@@ -502,12 +502,12 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>09:37</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -525,12 +525,12 @@
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>09:37</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -552,12 +552,12 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>09:37</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -575,12 +575,12 @@
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>09:37</t>
         </is>
       </c>
       <c r="F5" t="n">

</xml_diff>

<commit_message>
embedding GUI in a qt application is possible
</commit_message>
<xml_diff>
--- a/monet/tests/TestData/control/feedback_test_db.xlsx
+++ b/monet/tests/TestData/control/feedback_test_db.xlsx
@@ -507,7 +507,7 @@
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>09:37</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -530,7 +530,7 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>09:37</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -557,7 +557,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>09:37</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -580,7 +580,7 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>09:37</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="F5" t="n">

</xml_diff>

<commit_message>
documentation and test fixes
</commit_message>
<xml_diff>
--- a/monet/tests/TestData/control/feedback_test_db.xlsx
+++ b/monet/tests/TestData/control/feedback_test_db.xlsx
@@ -502,12 +502,12 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>17:07</t>
+          <t>13:54</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -525,12 +525,12 @@
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>17:07</t>
+          <t>13:54</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -552,12 +552,12 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>17:07</t>
+          <t>13:54</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -575,12 +575,12 @@
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>17:07</t>
+          <t>13:54</t>
         </is>
       </c>
       <c r="F5" t="n">

</xml_diff>